<commit_message>
Modification étude de marché
</commit_message>
<xml_diff>
--- a/étude_de_marché.xlsx
+++ b/étude_de_marché.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
   <si>
     <t>Nom</t>
   </si>
@@ -45,6 +45,9 @@
     <t xml:space="preserve">Fonctionnalités (résumé)</t>
   </si>
   <si>
+    <t xml:space="preserve">RELAIS + PRISE</t>
+  </si>
+  <si>
     <t xml:space="preserve">Shelly Plus 1</t>
   </si>
   <si>
@@ -115,6 +118,15 @@
   </si>
   <si>
     <t xml:space="preserve">Version compacte, MQTT natif, TLS + certificats, idéal si il y a peu de place (courant max plus faible)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EIGHTREE Prise tasmota</t>
+  </si>
+  <si>
+    <t>Amazon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prise Connectée WiFi, Compatible avec Home Assistant, MQTT, Domoticz, OpenHAB, ioBroker, 16A, 2,4 GHz Wi-Fi, 16A 3680W, 2PCS</t>
   </si>
   <si>
     <t>PARTICULES</t>
@@ -181,7 +193,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00\ [$€-40C]"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -191,9 +203,21 @@
     <font>
       <b/>
       <sz val="11.000000"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11.000000"/>
+      <color rgb="FF0F1111"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -205,17 +229,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="0"/>
-        <bgColor theme="0" tint="0"/>
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left style="none"/>
       <right style="none"/>
       <top style="none"/>
       <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
       <diagonal style="none"/>
     </border>
     <border>
@@ -228,30 +267,49 @@
       <top style="thin">
         <color theme="1"/>
       </top>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom style="thin">
-        <color theme="1"/>
+        <color auto="1"/>
       </bottom>
       <diagonal style="none"/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="1" fillId="2" borderId="1" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="2" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf fontId="2" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="3" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="3" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Output" xfId="1" builtinId="21"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -264,8 +322,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" displayName="Tableau1" ref="A1:I15">
-  <autoFilter ref="A1:I15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" displayName="Tableau1" ref="A1:I16">
+  <autoFilter ref="A1:I16"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Nom"/>
     <tableColumn id="2" name="Prix (EUR)"/>
@@ -277,7 +335,7 @@
     <tableColumn id="8" name="Relais / contact"/>
     <tableColumn id="9" name="Fonctionnalités (résumé)"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -735,7 +793,7 @@
     <col bestFit="1" min="6" max="6" width="18.28125"/>
     <col customWidth="1" min="7" max="7" width="20.28125"/>
     <col customWidth="1" min="8" max="8" width="19.421875"/>
-    <col customWidth="1" min="9" max="9" width="84.7109375"/>
+    <col customWidth="1" min="9" max="9" width="113.140625"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -768,288 +826,322 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="5"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="5">
         <v>16.489999999999998</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="C3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="D3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="E3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="F3" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="G3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="H3" s="6" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="s">
+      <c r="I3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="3">
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="5">
         <v>17.899999999999999</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="2" t="s">
+      <c r="C4" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="D4" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="E4" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="F4" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="G4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="H4" s="6" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="s">
+      <c r="I4" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="3">
+    </row>
+    <row r="5" ht="14.25">
+      <c r="A5" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="5">
         <v>15.35</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="C5" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="D5" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="E5" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="F5" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="G5" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="H5" s="6" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="5" ht="14.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
+      <c r="I5" s="6" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="6" ht="14.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
+      <c r="A6" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="5">
+        <v>24.989999999999998</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="7" ht="14.25">
-      <c r="A7" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
+      <c r="A7" s="6"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
     </row>
     <row r="8" ht="14.25">
-      <c r="A8" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B8" s="3">
+      <c r="A8" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="5"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+    </row>
+    <row r="9" ht="14.25">
+      <c r="A9" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" s="5">
         <v>47.700000000000003</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" ht="14.25">
-      <c r="A9" s="2" t="s">
+      <c r="C9" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="6">
+      <c r="D9" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" ht="14.25">
+      <c r="A10" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" s="5">
         <v>34.950000000000003</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="I9" s="5" t="s">
+      <c r="C10" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="H10" s="6" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="10" ht="14.25">
-      <c r="A10" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B10" s="3">
+      <c r="I10" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" ht="14.25">
+      <c r="A11" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B11" s="5">
         <v>174.09999999999999</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="11" ht="14.25">
-      <c r="A11" s="2"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
+      <c r="C11" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="12" ht="14.25">
-      <c r="A12" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
     </row>
     <row r="13" ht="14.25">
-      <c r="A13" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B13" s="3">
+      <c r="A13" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B13" s="5"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+    </row>
+    <row r="14" ht="14.25">
+      <c r="A14" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" s="5">
         <v>12.9</v>
       </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="14" ht="14.25">
-      <c r="A14" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B14" s="3">
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15" ht="14.25">
+      <c r="A15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B15" s="5">
         <v>17.5</v>
       </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="15" ht="14.25">
-      <c r="A15" s="8">
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
+      <c r="I15" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16" ht="14.25">
+      <c r="A16" s="9">
         <v>101020634</v>
       </c>
-      <c r="B15" s="3">
+      <c r="B16" s="5">
         <v>59.899999999999999</v>
       </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" ht="14.25">
+      <c r="I18" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>